<commit_message>
Add Graduated Enrolment Funnel and update cohort color specifications in HEMP Dashboard
</commit_message>
<xml_diff>
--- a/HEMP_Dashboard_Updated.xlsx
+++ b/HEMP_Dashboard_Updated.xlsx
@@ -975,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1180,142 +1180,10 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>DATA AGGREGATION</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Health Interest Areas</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Digital Health</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>[Value]</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Chart displays</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Mental Health</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>[Value]</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Chart displays</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Maternal &amp; Child Health</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>[Value]</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Chart displays</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Infectious Diseases</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>[Value]</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Chart displays</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Non-Communicable Diseases</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>[Value]</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Chart displays</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Health Systems</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>[Value]</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Chart displays</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1461,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1623,122 +1491,6 @@
       <c r="C11" s="5" t="inlineStr">
         <is>
           <t>✓ Consistent</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Font Weight</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Updated to 500</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>✓ Updated</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Placement Data by Programme:</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr"/>
-      <c r="C14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>BSc Software Engineering</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>95 placements</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>BSc Entrepreneurial Leadership</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>92 placements</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>ALURW - IBT</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>38 placements</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>ALCHE Variants</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>6 placements</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Included</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Teach-out Variants</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>9 placements</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Included</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1859,45 +1611,6 @@
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>10px</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Colour - Primary</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>#122B5E</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Colour - Secondary</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>#9FB4E0</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>✓ Added/Updated</t>
         </is>
       </c>
     </row>
@@ -1916,18 +1629,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>COURSES</t>
+          <t>COURSES - Graduated Enrolment Funnel</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1939,7 +1652,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>CHANGES MADE</t>
+          <t>COMPLETION JOURNEY TRACKING</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1951,12 +1664,12 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1968,124 +1681,511 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Participants by Health Interest Area</t>
+          <t>Enrolled</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>REMOVED</t>
+          <t>Total students starting course</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>✓ Deleted</t>
+          <t>KPI 1</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Streamline course-specific focus</t>
+          <t>Students finishing coursework</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Chart simplified</t>
+          <t>KPI 2</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Graduated</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Students completing all requirements</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>KPI 3</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Remaining Sections:</t>
-        </is>
-      </c>
+      <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr"/>
       <c r="C7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Enrolment &amp; Outcomes</t>
+          <t>Graduation Rate %</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Active - focus on programmes</t>
+          <t>(Graduated / Enrolled) × 100</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>✓ Updated</t>
+          <t>Key Metric</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Academic Performance</t>
+          <t>Completion Rate %</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Maintained</t>
+          <t>(Completed / Enrolled) × 100</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>✓ Keep</t>
+          <t>Key Metric</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Student Feedback</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Maintained</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>✓ Keep</t>
-        </is>
-      </c>
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Funnel Visualization</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Stage-by-stage progression</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Note:</t>
+          <t>Filter Options</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>All other course charts remain unchanged</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
+          <t>Year, Cohort, Programme</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Interactive</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>CHANGES MADE</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Previous</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Certification Metric</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Certified (single metric)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Graduated Enrolment Funnel</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>✓ Replaced</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Health Interest Chart</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Participants by HI</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>REMOVED</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>✓ Deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Chart Type</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Bar chart</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Funnel chart</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>✓ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Data Tracked</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Pass/Fail only</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Enrolled → Completed → Graduated</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>✓ Enhanced</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Visualization</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Single point metric</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Three-stage progression</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>✓ Improved</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>CHART SPECIFICATIONS: GRADUATED ENROLMENT FUNNEL</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Chart Type</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Funnel Chart</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Three-stage progression</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Enrolled</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Total students entering programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Students finishing coursework</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Graduated</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Students meeting all requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Year Filter</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>All Years, 2021, 2022, 2023, 2024, 2025, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Programme Filter</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>BSE, BEL, IBT, ALCHE, Teach-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="5" t="inlineStr"/>
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Primary Colour</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>#14306B</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Dark Navy</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Secondary Colour</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>#479BD6</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Light Blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Font Size (Labels)</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>10px</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Stage names</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Font Size (Numbers)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>11px</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Count values</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Data Labels</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Both Count &amp; %</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Show progression percentage</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2097,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2193,60 +2293,60 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Margins (top)</t>
+          <t>Font Size</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10px</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Margins (bottom)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="inlineStr"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Academic Programmes Charts</t>
+        </is>
+      </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Font Size</t>
+          <t>YAxis Width</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>10px</t>
+          <t>210px</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr"/>
-      <c r="C10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Margins (left)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Academic Programmes Charts</t>
-        </is>
-      </c>
+      <c r="A11" s="5" t="inlineStr"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>YAxis Width</t>
+          <t>Margins (right)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>210px</t>
+          <t>50</t>
         </is>
       </c>
     </row>
@@ -2254,38 +2354,34 @@
       <c r="A12" s="5" t="inlineStr"/>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Margins (left)</t>
+          <t>Font Size</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10px</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Margins (right)</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="B13" s="5" t="inlineStr"/>
+      <c r="C13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="5" t="inlineStr"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Graduated Enrolment Funnel</t>
+        </is>
+      </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Margins (top)</t>
+          <t>Chart Type</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Funnel</t>
         </is>
       </c>
     </row>
@@ -2293,12 +2389,12 @@
       <c r="A15" s="5" t="inlineStr"/>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Margins (bottom)</t>
+          <t>Stages</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3 (Enrolled, Completed, Graduated)</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2402,12 @@
       <c r="A16" s="5" t="inlineStr"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Font Size</t>
+          <t>Data Labels</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>10px</t>
+          <t>Count &amp; Percentage</t>
         </is>
       </c>
     </row>
@@ -2319,428 +2415,19 @@
       <c r="A17" s="5" t="inlineStr"/>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>Colour</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>210px accommodates full names</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>COLOUR PALETTE</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Element</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Hex Code</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Primary Brand</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>#14306B</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Dark Navy Blue</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Secondary Brand</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>#0C447C</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Darker Navy</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Accent</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>#479BD6</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Light Blue</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Health Interest Primary</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>#122B5E</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Deep Navy</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Health Interest Secondary</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>#9FB4E0</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Light Blue</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Text Primary</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>#6B7280</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Dark Grey</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Text Secondary</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>#9CA3AF</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Medium Grey</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Border</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>#D1D5DB</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Light Grey</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Background</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>#F3F4F6</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Very Light Grey</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>FONT STANDARDS</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="3" t="n"/>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Element</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Usage</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Chart Labels</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>10px</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Programme/Area names</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Percentages</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>9px</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Gender %, values</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Programme Text</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>8px</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>BSE, BEL, IBT breakdown</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Headers</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>12px</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Section headers</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Subheaders</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>11px</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Subsection headers</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>FILTERING STANDARDS</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="3" t="n"/>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>Chart Type</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Filter Available</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Options</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Health Interest</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>All Years, 2021, 2022, 2023, 2024, 2025, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Academic Programmes</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>All Years, 2021, 2022, 2023, 2024, 2025, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>All Years</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Always start with complete dataset</t>
+          <t>Brand Blue Gradient</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A39:F39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2752,7 +2439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2822,7 +2509,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Career Dev: Rename charts</t>
+          <t>Career Dev: Add health interest chart</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -2832,14 +2519,14 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Match new naming conventions</t>
+          <t>Year filter enabled</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Career Dev: Add health interest chart</t>
+          <t>Exposure Events: Add 2 charts side-by-side</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -2849,14 +2536,14 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Year filter enabled</t>
+          <t>Layout adjustment</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Career Dev: Position charts side-by-side</t>
+          <t>Internships: Remove Female Participation Trend</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -2866,14 +2553,14 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Same row layout</t>
+          <t>Delete chart</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Career Dev: Apply new styling</t>
+          <t>Internships: Update chart styling</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -2883,14 +2570,14 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Dimensions and colours</t>
+          <t>YAxis 210px</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Exposure Events: Add health interest chart</t>
+          <t>SIE: Add/update health interest chart</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -2907,7 +2594,7 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Exposure Events: Add academic programmes chart</t>
+          <t>Courses: Remove health interest chart</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -2917,14 +2604,14 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Year filter enabled</t>
+          <t>Delete chart</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Exposure Events: Position side-by-side</t>
+          <t>Courses: Replace Certified with Graduated Funnel</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -2934,14 +2621,14 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Same row layout</t>
+          <t>NEW - Key update</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Internships: Remove Female Participation Trend</t>
+          <t>Courses: Create funnel chart (Enrolled→Completed→Graduated)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -2951,14 +2638,14 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Delete chart</t>
+          <t>Three-stage visualization</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Internships: Move Placements chart</t>
+          <t>Courses: Add year and programme filters to funnel</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -2968,14 +2655,14 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Move to Student Feedback section</t>
+          <t>Interactive features</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Internships: Update chart styling</t>
+          <t>Apply colour standards</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -2985,14 +2672,14 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>YAxis 210px, new margins</t>
+          <t>All sheets</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>SIE: Add/update health interest chart</t>
+          <t>Apply font standards</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -3002,14 +2689,14 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Year filter enabled</t>
+          <t>All sheets</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>SIE: Apply styling</t>
+          <t>Test all charts display properly</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -3019,14 +2706,14 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>YAxis 130px, new margins</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Courses: Remove health interest chart</t>
+          <t>Verify all year filters functional</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -3036,14 +2723,14 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Delete chart</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Apply colour standards</t>
+          <t>Final review</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -3053,75 +2740,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>All sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Apply font standards</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>[ ] To Do</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>All sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Verify year filters functional</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>[ ] To Do</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Test each chart</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Test chart display</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>[ ] To Do</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Check dimensions, readability</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Final review</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>[ ] To Do</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Ensure all updates applied</t>
+          <t>Sign-off</t>
         </is>
       </c>
     </row>

</xml_diff>